<commit_message>
docs: update literature review tracking spreadsheet (v0.2)
</commit_message>
<xml_diff>
--- a/2026 MPV Literaturcheck v0.2 pasc.xlsx
+++ b/2026 MPV Literaturcheck v0.2 pasc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dxych-my.sharepoint.com/personal/pascalschmid_dxy_ch/Documents/Kunden/fxyz/SHP/Masterarbeit Vertiefung OneDrive/MPV/26-MPV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D296664-0C7B-4FE8-B352-6150EC47B447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="285" documentId="8_{1D296664-0C7B-4FE8-B352-6150EC47B447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CBBAAC5-8E32-B54B-85A3-7C00409153C0}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{FBD5382E-A212-41E0-9A0C-43789FF61CA2}"/>
+    <workbookView xWindow="1840" yWindow="5920" windowWidth="29400" windowHeight="18460" xr2:uid="{FBD5382E-A212-41E0-9A0C-43789FF61CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Literatur" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="321">
   <si>
     <t>Frage</t>
   </si>
@@ -223,9 +223,6 @@
     <t>Helle Köpfe mit Migrationshintergrund</t>
   </si>
   <si>
-    <t>XXX--XXX</t>
-  </si>
-  <si>
     <t>Seitenbereich aus Huser (2021) nachschlagen und in .bib eintragen</t>
   </si>
   <si>
@@ -767,13 +764,259 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7--52 </t>
+  </si>
+  <si>
+    <t>76-- 78</t>
+  </si>
+  <si>
+    <t>27--77</t>
+  </si>
+  <si>
+    <t>Grossenbacher und Tettenborn</t>
+  </si>
+  <si>
+    <t>1. Auflage</t>
+  </si>
+  <si>
+    <t>317--324</t>
+  </si>
+  <si>
+    <t>Handbuch Talententwicklung begabte Underachiever</t>
+  </si>
+  <si>
+    <t>Sparfeldt, Buch, Rost</t>
+  </si>
+  <si>
+    <t>365-372</t>
+  </si>
+  <si>
+    <t>Handbuch Talententwicklung Minoritäten als Begabungsreserven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">375-382 </t>
+  </si>
+  <si>
+    <t>Fischer und Fischer-Ontrup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handbuch Talententwicklung Begabung, Talent und Lern und leistungsschwierigkeiten </t>
+  </si>
+  <si>
+    <t>393-400</t>
+  </si>
+  <si>
+    <t>Sliwka</t>
+  </si>
+  <si>
+    <t>Handbuch Talententwicklung Die Bedeutung von Lehrkräften bei der Talentidentifikation und Förderung</t>
+  </si>
+  <si>
+    <t>453-462</t>
+  </si>
+  <si>
+    <t>Kaufmann und Gyssler</t>
+  </si>
+  <si>
+    <t>Sprachbegabung, Lesekompetenz und ihre Férderung in der Schulpraxis</t>
+  </si>
+  <si>
+    <t>487- 494</t>
+  </si>
+  <si>
+    <t>21--43</t>
+  </si>
+  <si>
+    <t>11--22</t>
+  </si>
+  <si>
+    <t>ca 4</t>
+  </si>
+  <si>
+    <t>Horvath2021EliteBegabung und soz Ungleichheit</t>
+  </si>
+  <si>
+    <t>Horvath</t>
+  </si>
+  <si>
+    <t>Elite, Begabung und soziale Ungleichheit- ungelöste Gerechtigskeitsfragen</t>
+  </si>
+  <si>
+    <t>77--85</t>
+  </si>
+  <si>
+    <t>Wollersheim2021 Handbuch Begabung</t>
+  </si>
+  <si>
+    <t>Wollersheim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Begabung als sozialhistorisches und soziokulturelles Konstrukt </t>
+  </si>
+  <si>
+    <t>88-99</t>
+  </si>
+  <si>
+    <t>Ziegler/Stern2021 Handbuch Begabung</t>
+  </si>
+  <si>
+    <t>Ziegler undStern</t>
+  </si>
+  <si>
+    <t>Der Einfluss von Erbe und Umwelt auf Bildung Intelligenz und Lernen</t>
+  </si>
+  <si>
+    <t>104-112</t>
+  </si>
+  <si>
+    <t>Stadelmann 2021</t>
+  </si>
+  <si>
+    <t>Stadelmann</t>
+  </si>
+  <si>
+    <t>Begbaungsentwicklung aus Sicht der Genetik und der kognitiven Neuropsychologie</t>
+  </si>
+  <si>
+    <t>133-147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Begabungsmodelle </t>
+  </si>
+  <si>
+    <t>204-219</t>
+  </si>
+  <si>
+    <t>Salome müller Oppliger 2021</t>
+  </si>
+  <si>
+    <t>Müller Oppliger</t>
+  </si>
+  <si>
+    <t>Pädagogische Diagnostik- Potenzialerfassung und Förderdiagnostik</t>
+  </si>
+  <si>
+    <t>224-235</t>
+  </si>
+  <si>
+    <t>Gauck2021Reimann</t>
+  </si>
+  <si>
+    <t>Gauck und Reimann</t>
+  </si>
+  <si>
+    <t>Psychologische Diagnostik in der Begabungd- und Begabtenförderung</t>
+  </si>
+  <si>
+    <t>239-249</t>
+  </si>
+  <si>
+    <t>Kuhn2021</t>
+  </si>
+  <si>
+    <t>Kuhl</t>
+  </si>
+  <si>
+    <t>Begabung,Bildung und Beziehung aus Sicht persönlchkeitspsychologisches Sicht</t>
+  </si>
+  <si>
+    <t>185-202</t>
+  </si>
+  <si>
+    <t>Reis,Renzulli,VMüllerOppliger</t>
+  </si>
+  <si>
+    <t>Das Schoolwide Enrichement Modell SEM</t>
+  </si>
+  <si>
+    <t>333-345</t>
+  </si>
+  <si>
+    <t>Stahl</t>
+  </si>
+  <si>
+    <t>Stahl2021</t>
+  </si>
+  <si>
+    <t>Das multidimensionale Begabungs-Entwicklungs-tool mBET als Instrument multifunktionaler Förderdiagnsotik</t>
+  </si>
+  <si>
+    <t>252-258</t>
+  </si>
+  <si>
+    <t>546-553</t>
+  </si>
+  <si>
+    <t>Greiten</t>
+  </si>
+  <si>
+    <t>Greiten 2021 Handbuch Begabung</t>
+  </si>
+  <si>
+    <t>Underachievement</t>
+  </si>
+  <si>
+    <t>stamm2021handbuchBegabung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">der fehlende Blick auf begabte Minoriäten </t>
+  </si>
+  <si>
+    <t>576-585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baum2021Schader Handbuch Begabung </t>
+  </si>
+  <si>
+    <t>Baum Schader</t>
+  </si>
+  <si>
+    <t>twice Exceptionality- in zweifacher Hinsicht aussergewöhnlich</t>
+  </si>
+  <si>
+    <t>588-598</t>
+  </si>
+  <si>
+    <t>121-123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Band 10 </t>
+  </si>
+  <si>
+    <t>Stärkung der Bildugnsgerechtigkeit bei Underachievement, Migration und Hochbegabung</t>
+  </si>
+  <si>
+    <t>fischer2020begabungsfoerderungWarnecke und Hauke</t>
+  </si>
+  <si>
+    <t>247--250</t>
+  </si>
+  <si>
+    <t>253--267</t>
+  </si>
+  <si>
+    <t>Koop Sedding2021</t>
+  </si>
+  <si>
+    <t>Koop Sedding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frühes Erkennen von hohen Begabungen </t>
+  </si>
+  <si>
+    <t>S. 260-267</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -801,6 +1044,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -838,7 +1088,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -854,11 +1104,191 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="30">
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1005,34 +1435,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}" name="Tabelle1" displayName="Tabelle1" ref="A5:R50" totalsRowShown="0" headerRowDxfId="13">
-  <autoFilter ref="A5:R50" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}" name="Tabelle1" displayName="Tabelle1" ref="A5:R72" totalsRowShown="0" headerRowDxfId="29">
+  <autoFilter ref="A5:R72" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{9388833E-F8F3-4B60-9392-969E617F4D54}" name="BibKey"/>
     <tableColumn id="2" xr3:uid="{1432EEC6-AA2F-4397-B85E-78BCD56BE3B5}" name="Frage"/>
     <tableColumn id="3" xr3:uid="{D9CE1E9B-5035-472D-A9F8-2F1033B994D7}" name="Autor:in"/>
-    <tableColumn id="4" xr3:uid="{1105A73B-730B-4281-9E3A-F8F53420E276}" name="Jahr" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{4980661F-8ADD-4EC9-915D-1FA21C36BDB5}" name="Titel (Kurz)" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{1105A73B-730B-4281-9E3A-F8F53420E276}" name="Jahr" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{4980661F-8ADD-4EC9-915D-1FA21C36BDB5}" name="Titel (Kurz)" dataDxfId="27"/>
     <tableColumn id="6" xr3:uid="{CCF50BC3-F643-43C7-BF90-47D076234654}" name="Werktyp"/>
     <tableColumn id="7" xr3:uid="{D612AC18-65F6-443E-9D0D-C75C308DFCF1}" name="Auflage"/>
     <tableColumn id="8" xr3:uid="{821F0CA5-D755-4F85-BC4A-104A0833BC19}" name="Seiten (bib)"/>
     <tableColumn id="9" xr3:uid="{3226AF62-8F66-48DA-A3AD-2941863A3434}" name="Seiten (verifiziert)"/>
-    <tableColumn id="10" xr3:uid="{488B9813-E2A6-4E52-AE1E-A5A3FE8E99AF}" name="Seiten-Status" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{488B9813-E2A6-4E52-AE1E-A5A3FE8E99AF}" name="Seiten-Status" dataDxfId="26"/>
     <tableColumn id="11" xr3:uid="{62484444-B9DF-4C6A-9465-DE3FDAA907CA}" name="Standort"/>
     <tableColumn id="12" xr3:uid="{D7CFB074-F68E-4E00-9BAF-29407CCE6462}" name="Signatur/URL"/>
-    <tableColumn id="13" xr3:uid="{BD05ABCA-4C13-42E4-B44D-7EBC8306F15A}" name="Prüfdatum" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{BD05ABCA-4C13-42E4-B44D-7EBC8306F15A}" name="Prüfdatum" dataDxfId="25"/>
     <tableColumn id="14" xr3:uid="{212484A1-2617-4C10-B87E-0108CCB285FF}" name="Prüfer:in-Kürzel"/>
     <tableColumn id="15" xr3:uid="{D855292C-D75F-4A74-BE97-306FEB67EAC1}" name="Im Dossier zitiert?"/>
     <tableColumn id="16" xr3:uid="{9749C062-563C-40B3-8131-1BF5F06E6EDA}" name="Kritische Felder"/>
-    <tableColumn id="17" xr3:uid="{BFDC7711-729C-4F0B-AA5F-027BE8104376}" name="Notiz" dataDxfId="8"/>
-    <tableColumn id="18" xr3:uid="{49B49761-C28F-4EA0-9FA6-57B2B50770C9}" name="Final OK" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{BFDC7711-729C-4F0B-AA5F-027BE8104376}" name="Notiz" dataDxfId="24"/>
+    <tableColumn id="18" xr3:uid="{49B49761-C28F-4EA0-9FA6-57B2B50770C9}" name="Final OK" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C9E7C783-D19A-4627-9CE4-C4F3C234CFB1}" name="Tabelle_Zitate" displayName="Tabelle_Zitate" ref="A1:C46" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C9E7C783-D19A-4627-9CE4-C4F3C234CFB1}" name="Tabelle_Zitate" displayName="Tabelle_Zitate" ref="A1:C46" totalsRowShown="0" headerRowDxfId="22">
   <autoFilter ref="A1:C46" xr:uid="{C9E7C783-D19A-4627-9CE4-C4F3C234CFB1}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{CEDA0375-43BE-42BD-8E91-B423FF614E66}" name="BibKey">
@@ -1389,7 +1819,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.5" customWidth="1"/>
@@ -1438,7 +1868,7 @@
       </c>
       <c r="B3" t="str">
         <f>COUNTIF(Tabelle1[Final OK],"✓") &amp; " / " &amp; ROWS(Tabelle1[])</f>
-        <v>0 / 45</v>
+        <v>0 / 67</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
@@ -1519,6 +1949,9 @@
       <c r="H6" t="s">
         <v>54</v>
       </c>
+      <c r="I6">
+        <v>10</v>
+      </c>
       <c r="J6" s="6" t="s">
         <v>21</v>
       </c>
@@ -1554,7 +1987,10 @@
         <v>14</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>241</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>21</v>
@@ -1567,13 +2003,13 @@
         <v>35</v>
       </c>
       <c r="Q7" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="R7" s="6"/>
     </row>
     <row r="8" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
@@ -1585,7 +2021,7 @@
         <v>2009</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F8" t="s">
         <v>17</v>
@@ -1601,25 +2037,25 @@
         <v>31</v>
       </c>
       <c r="Q8" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="R8" s="6"/>
     </row>
     <row r="9" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D9" s="6">
         <v>2018</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F9" t="s">
         <v>13</v>
@@ -1635,28 +2071,34 @@
         <v>31</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="R9" s="6"/>
     </row>
     <row r="10" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D10" s="6">
         <v>2013</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F10" t="s">
         <v>13</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="I10">
+        <v>46</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>22</v>
@@ -1669,25 +2111,25 @@
         <v>31</v>
       </c>
       <c r="Q10" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R10" s="6"/>
     </row>
     <row r="11" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D11" s="6">
         <v>2021</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F11" t="s">
         <v>13</v>
@@ -1703,31 +2145,37 @@
         <v>31</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R11" s="6"/>
     </row>
     <row r="12" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" s="6">
         <v>2016</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>79</v>
+        <v>78</v>
+      </c>
+      <c r="H12" t="s">
+        <v>242</v>
+      </c>
+      <c r="I12">
+        <v>40</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>22</v>
@@ -1740,28 +2188,34 @@
         <v>31</v>
       </c>
       <c r="Q12" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R12" s="6"/>
     </row>
     <row r="13" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D13" s="6">
         <v>2015</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F13" t="s">
         <v>13</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="I13">
+        <v>12</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>22</v>
@@ -1774,28 +2228,34 @@
         <v>31</v>
       </c>
       <c r="Q13" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R13" s="6"/>
     </row>
     <row r="14" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B14" t="s">
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D14" s="6">
         <v>2009</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
         <v>13</v>
+      </c>
+      <c r="H14" t="s">
+        <v>260</v>
+      </c>
+      <c r="I14">
+        <v>23</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>22</v>
@@ -1808,25 +2268,25 @@
         <v>31</v>
       </c>
       <c r="Q14" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R14" s="6"/>
     </row>
     <row r="15" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D15" s="6">
         <v>2012</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -1842,25 +2302,25 @@
         <v>31</v>
       </c>
       <c r="Q15" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R15" s="6"/>
     </row>
     <row r="16" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D16" s="6">
         <v>2014</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F16" t="s">
         <v>13</v>
@@ -1876,31 +2336,31 @@
         <v>31</v>
       </c>
       <c r="Q16" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="R16" s="6"/>
     </row>
     <row r="17" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B17" t="s">
         <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D17" s="6">
         <v>2020</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F17" t="s">
         <v>13</v>
       </c>
       <c r="G17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>22</v>
@@ -1913,31 +2373,31 @@
         <v>31</v>
       </c>
       <c r="Q17" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="R17" s="6"/>
     </row>
     <row r="18" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D18" s="6">
         <v>2010</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F18" t="s">
         <v>13</v>
       </c>
       <c r="G18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>22</v>
@@ -1950,31 +2410,31 @@
         <v>31</v>
       </c>
       <c r="Q18" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="R18" s="6"/>
     </row>
     <row r="19" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" t="s">
         <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" s="6">
         <v>2018</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
         <v>13</v>
       </c>
       <c r="G19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>22</v>
@@ -1987,25 +2447,25 @@
         <v>31</v>
       </c>
       <c r="Q19" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R19" s="6"/>
     </row>
     <row r="20" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D20" s="6">
         <v>2017</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F20" t="s">
         <v>13</v>
@@ -2021,28 +2481,37 @@
         <v>31</v>
       </c>
       <c r="Q20" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="R20" s="6"/>
     </row>
     <row r="21" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
         <v>113</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" t="s">
-        <v>114</v>
       </c>
       <c r="D21" s="6">
         <v>2020</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F21" t="s">
         <v>13</v>
+      </c>
+      <c r="G21" t="s">
+        <v>312</v>
+      </c>
+      <c r="H21" t="s">
+        <v>316</v>
+      </c>
+      <c r="I21">
+        <v>15</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>22</v>
@@ -2055,31 +2524,31 @@
         <v>31</v>
       </c>
       <c r="Q21" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R21" s="6"/>
     </row>
     <row r="22" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B22" t="s">
         <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D22" s="6">
         <v>2016</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="H22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>22</v>
@@ -2092,31 +2561,31 @@
         <v>31</v>
       </c>
       <c r="Q22" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="R22" s="6"/>
     </row>
     <row r="23" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B23" t="s">
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D23" s="6">
         <v>2010</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F23" t="s">
         <v>14</v>
       </c>
       <c r="H23" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>22</v>
@@ -2129,31 +2598,31 @@
         <v>31</v>
       </c>
       <c r="Q23" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="R23" s="6"/>
     </row>
     <row r="24" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D24" s="6">
         <v>2019</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
       </c>
       <c r="H24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>21</v>
@@ -2166,31 +2635,31 @@
         <v>35</v>
       </c>
       <c r="Q24" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="R24" s="6"/>
     </row>
     <row r="25" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D25" s="6">
         <v>2019</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F25" t="s">
         <v>14</v>
       </c>
       <c r="H25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>22</v>
@@ -2203,31 +2672,31 @@
         <v>31</v>
       </c>
       <c r="Q25" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="R25" s="6"/>
     </row>
     <row r="26" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D26" s="6">
         <v>2019</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F26" t="s">
         <v>13</v>
       </c>
       <c r="G26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>22</v>
@@ -2240,13 +2709,13 @@
         <v>31</v>
       </c>
       <c r="Q26" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="R26" s="6"/>
     </row>
     <row r="27" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
@@ -2258,7 +2727,7 @@
         <v>2012</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F27" t="s">
         <v>13</v>
@@ -2274,31 +2743,34 @@
         <v>31</v>
       </c>
       <c r="Q27" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="R27" s="6"/>
     </row>
     <row r="28" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D28" s="6">
         <v>2010</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="H28" t="s">
-        <v>147</v>
+        <v>146</v>
+      </c>
+      <c r="I28">
+        <v>14</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>22</v>
@@ -2311,25 +2783,25 @@
         <v>31</v>
       </c>
       <c r="Q28" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="R28" s="6"/>
     </row>
     <row r="29" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B29" t="s">
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D29" s="6">
         <v>2010</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F29" t="s">
         <v>13</v>
@@ -2345,31 +2817,31 @@
         <v>31</v>
       </c>
       <c r="Q29" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="R29" s="6"/>
     </row>
     <row r="30" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B30" t="s">
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D30" s="6">
         <v>2021</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="H30" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J30" s="6" t="s">
         <v>22</v>
@@ -2382,31 +2854,34 @@
         <v>31</v>
       </c>
       <c r="Q30" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R30" s="6"/>
     </row>
     <row r="31" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>157</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
         <v>158</v>
-      </c>
-      <c r="B31" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" t="s">
-        <v>159</v>
       </c>
       <c r="D31" s="6">
         <v>2021</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F31" t="s">
         <v>14</v>
       </c>
       <c r="H31" t="s">
-        <v>161</v>
+        <v>160</v>
+      </c>
+      <c r="I31">
+        <v>11</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>22</v>
@@ -2419,31 +2894,31 @@
         <v>31</v>
       </c>
       <c r="Q31" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R31" s="6"/>
     </row>
     <row r="32" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B32" t="s">
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D32" s="6">
         <v>2021</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="H32" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J32" s="6" t="s">
         <v>22</v>
@@ -2456,25 +2931,25 @@
         <v>31</v>
       </c>
       <c r="Q32" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R32" s="6"/>
     </row>
     <row r="33" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B33" t="s">
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D33" s="6">
         <v>2010</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F33" t="s">
         <v>17</v>
@@ -2490,31 +2965,31 @@
         <v>31</v>
       </c>
       <c r="Q33" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R33" s="6"/>
     </row>
     <row r="34" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B34" t="s">
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D34" s="6">
         <v>2021</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F34" t="s">
         <v>13</v>
       </c>
       <c r="G34" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J34" s="6" t="s">
         <v>21</v>
@@ -2527,31 +3002,31 @@
         <v>32</v>
       </c>
       <c r="Q34" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="R34" s="6"/>
     </row>
     <row r="35" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B35" t="s">
         <v>11</v>
       </c>
       <c r="C35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D35" s="6">
         <v>2021</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F35" t="s">
         <v>13</v>
       </c>
       <c r="G35" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J35" s="6" t="s">
         <v>22</v>
@@ -2564,25 +3039,25 @@
         <v>31</v>
       </c>
       <c r="Q35" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="R35" s="6"/>
     </row>
     <row r="36" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B36" t="s">
         <v>11</v>
       </c>
       <c r="C36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D36" s="6">
         <v>2020</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F36" t="s">
         <v>13</v>
@@ -2598,25 +3073,25 @@
         <v>31</v>
       </c>
       <c r="Q36" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="R36" s="6"/>
     </row>
     <row r="37" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B37" t="s">
         <v>11</v>
       </c>
       <c r="C37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D37" s="6">
         <v>2021</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F37" t="s">
         <v>17</v>
@@ -2632,25 +3107,25 @@
         <v>31</v>
       </c>
       <c r="Q37" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R37" s="6"/>
     </row>
     <row r="38" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B38" t="s">
         <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D38" s="6">
         <v>2021</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F38" t="s">
         <v>13</v>
@@ -2666,31 +3141,31 @@
         <v>31</v>
       </c>
       <c r="Q38" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="R38" s="6"/>
     </row>
     <row r="39" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B39" t="s">
         <v>11</v>
       </c>
       <c r="C39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D39" s="6">
         <v>2019</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
       <c r="H39" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J39" s="6" t="s">
         <v>21</v>
@@ -2703,25 +3178,25 @@
         <v>35</v>
       </c>
       <c r="Q39" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="R39" s="6"/>
     </row>
     <row r="40" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B40" t="s">
         <v>12</v>
       </c>
       <c r="C40" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D40" s="6">
         <v>2022</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F40" t="s">
         <v>18</v>
@@ -2737,25 +3212,25 @@
         <v>31</v>
       </c>
       <c r="Q40" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="R40" s="6"/>
     </row>
     <row r="41" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B41" t="s">
         <v>12</v>
       </c>
       <c r="C41" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D41" s="6">
         <v>2023</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F41" t="s">
         <v>18</v>
@@ -2771,25 +3246,25 @@
         <v>31</v>
       </c>
       <c r="Q41" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="R41" s="6"/>
     </row>
     <row r="42" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B42" t="s">
         <v>12</v>
       </c>
       <c r="C42" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D42" s="6">
         <v>2014</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F42" t="s">
         <v>13</v>
@@ -2805,28 +3280,31 @@
         <v>31</v>
       </c>
       <c r="Q42" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="R42" s="6"/>
     </row>
     <row r="43" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B43" t="s">
         <v>12</v>
       </c>
       <c r="C43" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D43" s="6">
         <v>2025</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F43" t="s">
         <v>15</v>
+      </c>
+      <c r="I43" t="s">
+        <v>262</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>22</v>
@@ -2839,13 +3317,13 @@
         <v>31</v>
       </c>
       <c r="Q43" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="R43" s="6"/>
     </row>
     <row r="44" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B44" t="s">
         <v>12</v>
@@ -2857,10 +3335,13 @@
         <v>2011</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F44" t="s">
         <v>16</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
       </c>
       <c r="J44" s="6" t="s">
         <v>22</v>
@@ -2873,28 +3354,31 @@
         <v>31</v>
       </c>
       <c r="Q44" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="R44" s="6"/>
     </row>
     <row r="45" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B45" t="s">
         <v>12</v>
       </c>
       <c r="C45" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D45" s="6">
         <v>2023</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F45" t="s">
         <v>16</v>
+      </c>
+      <c r="I45">
+        <v>4</v>
       </c>
       <c r="J45" s="6" t="s">
         <v>22</v>
@@ -2907,25 +3391,25 @@
         <v>31</v>
       </c>
       <c r="Q45" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="R45" s="6"/>
     </row>
     <row r="46" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B46" t="s">
         <v>12</v>
       </c>
       <c r="C46" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D46" s="6">
         <v>2025</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F46" t="s">
         <v>16</v>
@@ -2941,31 +3425,31 @@
         <v>31</v>
       </c>
       <c r="Q46" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="R46" s="6"/>
     </row>
     <row r="47" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B47" t="s">
         <v>7</v>
       </c>
       <c r="C47" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D47" s="6">
         <v>2020</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F47" t="s">
         <v>15</v>
       </c>
       <c r="H47" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J47" s="6" t="s">
         <v>22</v>
@@ -2978,31 +3462,31 @@
         <v>31</v>
       </c>
       <c r="Q47" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="R47" s="6"/>
     </row>
     <row r="48" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B48" t="s">
         <v>7</v>
       </c>
       <c r="C48" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D48" s="6">
         <v>2020</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F48" t="s">
         <v>15</v>
       </c>
       <c r="H48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J48" s="6" t="s">
         <v>22</v>
@@ -3015,31 +3499,31 @@
         <v>31</v>
       </c>
       <c r="Q48" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="R48" s="6"/>
     </row>
     <row r="49" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B49" t="s">
         <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D49" s="6">
         <v>2021</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F49" t="s">
         <v>15</v>
       </c>
       <c r="H49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J49" s="6" t="s">
         <v>22</v>
@@ -3052,25 +3536,25 @@
         <v>31</v>
       </c>
       <c r="Q49" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="R49" s="6"/>
     </row>
     <row r="50" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B50" t="s">
         <v>7</v>
       </c>
       <c r="C50" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D50" s="6">
         <v>2025</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F50" t="s">
         <v>15</v>
@@ -3086,23 +3570,778 @@
         <v>31</v>
       </c>
       <c r="Q50" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="R50" s="6"/>
     </row>
+    <row r="51" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A51" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B51" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" t="s">
+        <v>243</v>
+      </c>
+      <c r="D51" s="6">
+        <v>2014</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F51" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" t="s">
+        <v>244</v>
+      </c>
+      <c r="H51" t="s">
+        <v>245</v>
+      </c>
+      <c r="I51">
+        <v>8</v>
+      </c>
+      <c r="J51" s="6"/>
+      <c r="M51" s="10"/>
+      <c r="Q51" s="8"/>
+      <c r="R51" s="6"/>
+    </row>
+    <row r="52" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A52" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" t="s">
+        <v>247</v>
+      </c>
+      <c r="D52" s="6">
+        <v>2014</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="F52" t="s">
+        <v>13</v>
+      </c>
+      <c r="H52" t="s">
+        <v>248</v>
+      </c>
+      <c r="I52">
+        <v>8</v>
+      </c>
+      <c r="J52" s="6"/>
+      <c r="M52" s="10"/>
+      <c r="Q52" s="8"/>
+      <c r="R52" s="6"/>
+    </row>
+    <row r="53" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A53" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" t="s">
+        <v>52</v>
+      </c>
+      <c r="D53" s="6">
+        <v>2014</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="F53" t="s">
+        <v>13</v>
+      </c>
+      <c r="H53" t="s">
+        <v>250</v>
+      </c>
+      <c r="I53">
+        <v>8</v>
+      </c>
+      <c r="J53" s="6"/>
+      <c r="M53" s="10"/>
+      <c r="Q53" s="8"/>
+      <c r="R53" s="6"/>
+    </row>
+    <row r="54" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A54" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>251</v>
+      </c>
+      <c r="D54" s="6">
+        <v>2014</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="F54" t="s">
+        <v>13</v>
+      </c>
+      <c r="H54" t="s">
+        <v>253</v>
+      </c>
+      <c r="I54">
+        <v>8</v>
+      </c>
+      <c r="J54" s="6"/>
+      <c r="M54" s="10"/>
+      <c r="Q54" s="8"/>
+      <c r="R54" s="6"/>
+    </row>
+    <row r="55" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A55" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C55" t="s">
+        <v>254</v>
+      </c>
+      <c r="D55" s="6">
+        <v>2014</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="F55" t="s">
+        <v>13</v>
+      </c>
+      <c r="H55" t="s">
+        <v>256</v>
+      </c>
+      <c r="I55">
+        <v>10</v>
+      </c>
+      <c r="J55" s="6"/>
+      <c r="M55" s="10"/>
+      <c r="Q55" s="8"/>
+      <c r="R55" s="6"/>
+    </row>
+    <row r="56" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A56" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" t="s">
+        <v>257</v>
+      </c>
+      <c r="D56" s="6">
+        <v>2014</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="F56" t="s">
+        <v>13</v>
+      </c>
+      <c r="H56" t="s">
+        <v>259</v>
+      </c>
+      <c r="I56">
+        <v>8</v>
+      </c>
+      <c r="J56" s="6"/>
+      <c r="M56" s="10"/>
+      <c r="Q56" s="8"/>
+      <c r="R56" s="6"/>
+    </row>
+    <row r="57" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A57" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="B57" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" t="s">
+        <v>264</v>
+      </c>
+      <c r="D57" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="F57" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" t="s">
+        <v>244</v>
+      </c>
+      <c r="H57" t="s">
+        <v>266</v>
+      </c>
+      <c r="I57">
+        <v>9</v>
+      </c>
+      <c r="J57" s="6"/>
+      <c r="M57" s="10"/>
+      <c r="Q57" s="8"/>
+      <c r="R57" s="6"/>
+    </row>
+    <row r="58" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A58" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" t="s">
+        <v>268</v>
+      </c>
+      <c r="D58" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58" t="s">
+        <v>244</v>
+      </c>
+      <c r="H58" t="s">
+        <v>270</v>
+      </c>
+      <c r="I58">
+        <v>12</v>
+      </c>
+      <c r="J58" s="6"/>
+      <c r="M58" s="10"/>
+      <c r="Q58" s="8"/>
+      <c r="R58" s="6"/>
+    </row>
+    <row r="59" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A59" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" t="s">
+        <v>272</v>
+      </c>
+      <c r="D59" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" t="s">
+        <v>244</v>
+      </c>
+      <c r="H59" t="s">
+        <v>274</v>
+      </c>
+      <c r="I59">
+        <v>8</v>
+      </c>
+      <c r="J59" s="6"/>
+      <c r="M59" s="10"/>
+      <c r="Q59" s="8"/>
+      <c r="R59" s="6"/>
+    </row>
+    <row r="60" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A60" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" t="s">
+        <v>276</v>
+      </c>
+      <c r="D60" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>244</v>
+      </c>
+      <c r="H60" t="s">
+        <v>278</v>
+      </c>
+      <c r="I60">
+        <v>14</v>
+      </c>
+      <c r="J60" s="6"/>
+      <c r="M60" s="10"/>
+      <c r="Q60" s="8"/>
+      <c r="R60" s="6"/>
+    </row>
+    <row r="61" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A61" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" t="s">
+        <v>162</v>
+      </c>
+      <c r="D61" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="F61" t="s">
+        <v>14</v>
+      </c>
+      <c r="G61" t="s">
+        <v>244</v>
+      </c>
+      <c r="H61" t="s">
+        <v>280</v>
+      </c>
+      <c r="I61">
+        <v>16</v>
+      </c>
+      <c r="J61" s="6"/>
+      <c r="M61" s="10"/>
+      <c r="Q61" s="8"/>
+      <c r="R61" s="6"/>
+    </row>
+    <row r="62" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A62" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" t="s">
+        <v>282</v>
+      </c>
+      <c r="D62" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>244</v>
+      </c>
+      <c r="H62" t="s">
+        <v>284</v>
+      </c>
+      <c r="I62">
+        <v>12</v>
+      </c>
+      <c r="J62" s="6"/>
+      <c r="M62" s="10"/>
+      <c r="Q62" s="8"/>
+      <c r="R62" s="6"/>
+    </row>
+    <row r="63" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A63" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>286</v>
+      </c>
+      <c r="D63" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="F63" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" t="s">
+        <v>244</v>
+      </c>
+      <c r="H63" t="s">
+        <v>288</v>
+      </c>
+      <c r="I63">
+        <v>11</v>
+      </c>
+      <c r="J63" s="6"/>
+      <c r="M63" s="10"/>
+      <c r="Q63" s="8"/>
+      <c r="R63" s="6"/>
+    </row>
+    <row r="64" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A64" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>290</v>
+      </c>
+      <c r="D64" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="F64" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64" t="s">
+        <v>244</v>
+      </c>
+      <c r="H64" t="s">
+        <v>292</v>
+      </c>
+      <c r="J64" s="6"/>
+      <c r="M64" s="10"/>
+      <c r="Q64" s="8"/>
+      <c r="R64" s="6"/>
+    </row>
+    <row r="65" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" t="s">
+        <v>293</v>
+      </c>
+      <c r="D65" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E65" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="F65" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65" t="s">
+        <v>244</v>
+      </c>
+      <c r="H65" t="s">
+        <v>295</v>
+      </c>
+      <c r="J65" s="6"/>
+      <c r="M65" s="10"/>
+      <c r="Q65" s="8"/>
+      <c r="R65" s="6"/>
+    </row>
+    <row r="66" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A66" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" t="s">
+        <v>296</v>
+      </c>
+      <c r="D66" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="F66" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66" t="s">
+        <v>244</v>
+      </c>
+      <c r="H66" t="s">
+        <v>299</v>
+      </c>
+      <c r="I66">
+        <v>7</v>
+      </c>
+      <c r="J66" s="6"/>
+      <c r="M66" s="10"/>
+      <c r="Q66" s="8"/>
+      <c r="R66" s="6"/>
+    </row>
+    <row r="67" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C67" t="s">
+        <v>301</v>
+      </c>
+      <c r="D67" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E67" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="F67" t="s">
+        <v>14</v>
+      </c>
+      <c r="G67" t="s">
+        <v>244</v>
+      </c>
+      <c r="H67" t="s">
+        <v>300</v>
+      </c>
+      <c r="J67" s="6"/>
+      <c r="M67" s="10"/>
+      <c r="Q67" s="8"/>
+      <c r="R67" s="6"/>
+    </row>
+    <row r="68" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C68" t="s">
+        <v>52</v>
+      </c>
+      <c r="D68" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E68" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="F68" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" t="s">
+        <v>244</v>
+      </c>
+      <c r="H68" t="s">
+        <v>306</v>
+      </c>
+      <c r="I68">
+        <v>10</v>
+      </c>
+      <c r="J68" s="6"/>
+      <c r="M68" s="10"/>
+      <c r="Q68" s="8"/>
+      <c r="R68" s="6"/>
+    </row>
+    <row r="69" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C69" t="s">
+        <v>308</v>
+      </c>
+      <c r="D69" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E69" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="F69" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" t="s">
+        <v>244</v>
+      </c>
+      <c r="H69" t="s">
+        <v>310</v>
+      </c>
+      <c r="I69">
+        <v>11</v>
+      </c>
+      <c r="J69" s="6"/>
+      <c r="M69" s="10"/>
+      <c r="Q69" s="8"/>
+      <c r="R69" s="6"/>
+    </row>
+    <row r="70" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A70" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>76</v>
+      </c>
+      <c r="D70" s="6">
+        <v>2016</v>
+      </c>
+      <c r="E70" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F70" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" t="s">
+        <v>78</v>
+      </c>
+      <c r="H70" t="s">
+        <v>311</v>
+      </c>
+      <c r="I70">
+        <v>3</v>
+      </c>
+      <c r="J70" s="6"/>
+      <c r="M70" s="10"/>
+      <c r="Q70" s="8"/>
+      <c r="R70" s="6"/>
+    </row>
+    <row r="71" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+      <c r="A71" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C71" t="s">
+        <v>113</v>
+      </c>
+      <c r="D71" s="6">
+        <v>2020</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="F71" t="s">
+        <v>13</v>
+      </c>
+      <c r="G71" t="s">
+        <v>312</v>
+      </c>
+      <c r="H71" t="s">
+        <v>315</v>
+      </c>
+      <c r="I71">
+        <v>4</v>
+      </c>
+      <c r="J71" s="6"/>
+      <c r="M71" s="10"/>
+      <c r="Q71" s="8"/>
+      <c r="R71" s="6"/>
+    </row>
+    <row r="72" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A72" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C72" t="s">
+        <v>318</v>
+      </c>
+      <c r="D72" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E72" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="F72" t="s">
+        <v>14</v>
+      </c>
+      <c r="G72" t="s">
+        <v>244</v>
+      </c>
+      <c r="H72" t="s">
+        <v>320</v>
+      </c>
+      <c r="I72">
+        <v>8</v>
+      </c>
+      <c r="J72" s="6"/>
+      <c r="M72" s="10"/>
+      <c r="Q72" s="8"/>
+      <c r="R72" s="6"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A6:R50">
-    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="A6:R9 A11:R11 A10:G10 A13:R50 A12:G12 I12:R12 J10:R10">
+    <cfRule type="expression" dxfId="21" priority="13" stopIfTrue="1">
       <formula>$R6="✓"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="20" priority="14">
       <formula>$O6="Nein"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="19" priority="15">
       <formula>$J6="TODO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="18" priority="16">
       <formula>$J6="Abweichung"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12:I12">
+    <cfRule type="expression" dxfId="17" priority="21" stopIfTrue="1">
+      <formula>$R10="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="22">
+      <formula>$O10="Nein"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="23">
+      <formula>$J10="TODO"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="24">
+      <formula>$J10="Abweichung"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A70">
+    <cfRule type="expression" dxfId="11" priority="9" stopIfTrue="1">
+      <formula>$R70="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="10">
+      <formula>$O70="Nein"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="11">
+      <formula>$J70="TODO"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="12">
+      <formula>$J70="Abweichung"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C71">
+    <cfRule type="expression" dxfId="7" priority="5" stopIfTrue="1">
+      <formula>$R71="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="6">
+      <formula>$O71="Nein"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="7">
+      <formula>$J71="TODO"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="8">
+      <formula>$J71="Abweichung"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A71">
+    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
+      <formula>$R71="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$O71="Nein"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="3">
+      <formula>$J71="TODO"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>$J71="Abweichung"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3117,43 +4356,43 @@
           <x14:formula1>
             <xm:f>Listen!$A$2:$A$7</xm:f>
           </x14:formula1>
-          <xm:sqref>B6:B50</xm:sqref>
+          <xm:sqref>B6:B72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Dropdown-Liste wählen." xr:uid="{22FB5F8D-6434-40FA-A338-F412E79D5A6D}">
           <x14:formula1>
             <xm:f>Listen!$B$2:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>F6:F50</xm:sqref>
+          <xm:sqref>F6:F72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Dropdown-Liste wählen." xr:uid="{7B3378E9-3663-4962-954C-2DE3FFD4F476}">
           <x14:formula1>
             <xm:f>Listen!$C$2:$C$5</xm:f>
           </x14:formula1>
-          <xm:sqref>J6:J50</xm:sqref>
+          <xm:sqref>J6:J72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Dropdown-Liste wählen." xr:uid="{261C7A44-F3B8-4148-9CF4-546DF5EA2F09}">
           <x14:formula1>
             <xm:f>Listen!$D$2:$D$6</xm:f>
           </x14:formula1>
-          <xm:sqref>K6:K50</xm:sqref>
+          <xm:sqref>K6:K72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Dropdown-Liste wählen." xr:uid="{2902D571-B10E-4AE1-8BD1-4A5FE6D0D192}">
           <x14:formula1>
             <xm:f>Listen!$E$2:$E$4</xm:f>
           </x14:formula1>
-          <xm:sqref>O6:O50</xm:sqref>
+          <xm:sqref>O6:O72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Dropdown-Liste wählen." xr:uid="{B10C74D7-995A-4A9C-915A-095DF0C6191C}">
           <x14:formula1>
             <xm:f>Listen!$F$2:$F$7</xm:f>
           </x14:formula1>
-          <xm:sqref>P6:P50</xm:sqref>
+          <xm:sqref>P6:P72</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Dropdown-Liste wählen." xr:uid="{1274EEF3-7C33-4D7B-B823-8B28782E9D15}">
           <x14:formula1>
             <xm:f>Listen!$G$2:$G$3</xm:f>
           </x14:formula1>
-          <xm:sqref>R6:R50</xm:sqref>
+          <xm:sqref>R6:R72</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3176,10 +4415,10 @@
         <v>43</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -3634,10 +4873,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C46">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>$C2="OK"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>$C2="NICHT ZITIERT"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
docs: add bibliography export tooling and generate CSV/XLSX literature overviews
</commit_message>
<xml_diff>
--- a/2026 MPV Literaturcheck v0.2 pasc.xlsx
+++ b/2026 MPV Literaturcheck v0.2 pasc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dxych-my.sharepoint.com/personal/pascalschmid_dxy_ch/Documents/Kunden/fxyz/SHP/Masterarbeit Vertiefung OneDrive/MPV/26-MPV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="285" documentId="8_{1D296664-0C7B-4FE8-B352-6150EC47B447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CBBAAC5-8E32-B54B-85A3-7C00409153C0}"/>
+  <xr:revisionPtr revIDLastSave="286" documentId="8_{1D296664-0C7B-4FE8-B352-6150EC47B447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D654531A-6443-4270-9B18-3884D2052CB4}"/>
   <bookViews>
-    <workbookView xWindow="1840" yWindow="5920" windowWidth="29400" windowHeight="18460" xr2:uid="{FBD5382E-A212-41E0-9A0C-43789FF61CA2}"/>
+    <workbookView xWindow="-35240" yWindow="9550" windowWidth="34940" windowHeight="15960" xr2:uid="{FBD5382E-A212-41E0-9A0C-43789FF61CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Literatur" sheetId="1" r:id="rId1"/>
@@ -1013,9 +1013,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1088,7 +1085,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1105,36 +1102,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
-    <dxf>
-      <font>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="26">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1220,28 +1193,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1386,7 +1337,7 @@
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -1435,34 +1386,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}" name="Tabelle1" displayName="Tabelle1" ref="A5:R72" totalsRowShown="0" headerRowDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}" name="Tabelle1" displayName="Tabelle1" ref="A5:R72" totalsRowShown="0" headerRowDxfId="25">
   <autoFilter ref="A5:R72" xr:uid="{8CB11F9B-92E3-44E8-AC7A-E53702FFAB53}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{9388833E-F8F3-4B60-9392-969E617F4D54}" name="BibKey"/>
     <tableColumn id="2" xr3:uid="{1432EEC6-AA2F-4397-B85E-78BCD56BE3B5}" name="Frage"/>
     <tableColumn id="3" xr3:uid="{D9CE1E9B-5035-472D-A9F8-2F1033B994D7}" name="Autor:in"/>
-    <tableColumn id="4" xr3:uid="{1105A73B-730B-4281-9E3A-F8F53420E276}" name="Jahr" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{4980661F-8ADD-4EC9-915D-1FA21C36BDB5}" name="Titel (Kurz)" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{1105A73B-730B-4281-9E3A-F8F53420E276}" name="Jahr" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{4980661F-8ADD-4EC9-915D-1FA21C36BDB5}" name="Titel (Kurz)" dataDxfId="23"/>
     <tableColumn id="6" xr3:uid="{CCF50BC3-F643-43C7-BF90-47D076234654}" name="Werktyp"/>
     <tableColumn id="7" xr3:uid="{D612AC18-65F6-443E-9D0D-C75C308DFCF1}" name="Auflage"/>
     <tableColumn id="8" xr3:uid="{821F0CA5-D755-4F85-BC4A-104A0833BC19}" name="Seiten (bib)"/>
     <tableColumn id="9" xr3:uid="{3226AF62-8F66-48DA-A3AD-2941863A3434}" name="Seiten (verifiziert)"/>
-    <tableColumn id="10" xr3:uid="{488B9813-E2A6-4E52-AE1E-A5A3FE8E99AF}" name="Seiten-Status" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{488B9813-E2A6-4E52-AE1E-A5A3FE8E99AF}" name="Seiten-Status" dataDxfId="22"/>
     <tableColumn id="11" xr3:uid="{62484444-B9DF-4C6A-9465-DE3FDAA907CA}" name="Standort"/>
     <tableColumn id="12" xr3:uid="{D7CFB074-F68E-4E00-9BAF-29407CCE6462}" name="Signatur/URL"/>
-    <tableColumn id="13" xr3:uid="{BD05ABCA-4C13-42E4-B44D-7EBC8306F15A}" name="Prüfdatum" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{BD05ABCA-4C13-42E4-B44D-7EBC8306F15A}" name="Prüfdatum" dataDxfId="21"/>
     <tableColumn id="14" xr3:uid="{212484A1-2617-4C10-B87E-0108CCB285FF}" name="Prüfer:in-Kürzel"/>
     <tableColumn id="15" xr3:uid="{D855292C-D75F-4A74-BE97-306FEB67EAC1}" name="Im Dossier zitiert?"/>
     <tableColumn id="16" xr3:uid="{9749C062-563C-40B3-8131-1BF5F06E6EDA}" name="Kritische Felder"/>
-    <tableColumn id="17" xr3:uid="{BFDC7711-729C-4F0B-AA5F-027BE8104376}" name="Notiz" dataDxfId="24"/>
-    <tableColumn id="18" xr3:uid="{49B49761-C28F-4EA0-9FA6-57B2B50770C9}" name="Final OK" dataDxfId="23"/>
+    <tableColumn id="17" xr3:uid="{BFDC7711-729C-4F0B-AA5F-027BE8104376}" name="Notiz" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{49B49761-C28F-4EA0-9FA6-57B2B50770C9}" name="Final OK" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C9E7C783-D19A-4627-9CE4-C4F3C234CFB1}" name="Tabelle_Zitate" displayName="Tabelle_Zitate" ref="A1:C46" totalsRowShown="0" headerRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C9E7C783-D19A-4627-9CE4-C4F3C234CFB1}" name="Tabelle_Zitate" displayName="Tabelle_Zitate" ref="A1:C46" totalsRowShown="0" headerRowDxfId="18">
   <autoFilter ref="A1:C46" xr:uid="{C9E7C783-D19A-4627-9CE4-C4F3C234CFB1}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{CEDA0375-43BE-42BD-8E91-B423FF614E66}" name="BibKey">
@@ -1478,7 +1429,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1794,7 +1745,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="5">
+  <wetp:taskpane dockstate="right" visibility="0" width="1153" row="5">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1820,28 +1771,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R72"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="35.5" customWidth="1"/>
-    <col min="2" max="2" width="12.5" customWidth="1"/>
+    <col min="1" max="1" width="35.46484375" customWidth="1"/>
+    <col min="2" max="2" width="12.46484375" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" customWidth="1"/>
-    <col min="5" max="5" width="49.83203125" customWidth="1"/>
-    <col min="6" max="6" width="23.1640625" customWidth="1"/>
-    <col min="7" max="7" width="14.1640625" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="10" width="19.5" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.796875" customWidth="1"/>
+    <col min="5" max="5" width="49.796875" customWidth="1"/>
+    <col min="6" max="6" width="23.1328125" customWidth="1"/>
+    <col min="7" max="7" width="14.1328125" customWidth="1"/>
+    <col min="8" max="8" width="16.796875" customWidth="1"/>
+    <col min="9" max="10" width="19.46484375" customWidth="1"/>
+    <col min="11" max="11" width="17.796875" customWidth="1"/>
+    <col min="12" max="12" width="24.796875" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="14.1640625" customWidth="1"/>
-    <col min="15" max="15" width="15.1640625" customWidth="1"/>
-    <col min="16" max="16" width="19.5" customWidth="1"/>
-    <col min="17" max="17" width="49.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.5" customWidth="1"/>
+    <col min="14" max="14" width="14.1328125" customWidth="1"/>
+    <col min="15" max="15" width="15.1328125" customWidth="1"/>
+    <col min="16" max="16" width="19.46484375" customWidth="1"/>
+    <col min="17" max="17" width="49.796875" customWidth="1"/>
+    <col min="18" max="18" width="12.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -1853,7 +1804,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
@@ -1862,7 +1813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
@@ -1871,7 +1822,7 @@
         <v>0 / 67</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
         <v>43</v>
       </c>
@@ -1927,7 +1878,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -1967,7 +1918,7 @@
       </c>
       <c r="R6" s="6"/>
     </row>
-    <row r="7" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>56</v>
       </c>
@@ -2007,7 +1958,7 @@
       </c>
       <c r="R7" s="6"/>
     </row>
-    <row r="8" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -2041,7 +1992,7 @@
       </c>
       <c r="R8" s="6"/>
     </row>
-    <row r="9" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -2075,7 +2026,7 @@
       </c>
       <c r="R9" s="6"/>
     </row>
-    <row r="10" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>67</v>
       </c>
@@ -2115,7 +2066,7 @@
       </c>
       <c r="R10" s="6"/>
     </row>
-    <row r="11" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -2149,7 +2100,7 @@
       </c>
       <c r="R11" s="6"/>
     </row>
-    <row r="12" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>75</v>
       </c>
@@ -2192,7 +2143,7 @@
       </c>
       <c r="R12" s="6"/>
     </row>
-    <row r="13" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>79</v>
       </c>
@@ -2232,7 +2183,7 @@
       </c>
       <c r="R13" s="6"/>
     </row>
-    <row r="14" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>83</v>
       </c>
@@ -2272,7 +2223,7 @@
       </c>
       <c r="R14" s="6"/>
     </row>
-    <row r="15" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -2306,7 +2257,7 @@
       </c>
       <c r="R15" s="6"/>
     </row>
-    <row r="16" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>91</v>
       </c>
@@ -2340,7 +2291,7 @@
       </c>
       <c r="R16" s="6"/>
     </row>
-    <row r="17" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>95</v>
       </c>
@@ -2377,7 +2328,7 @@
       </c>
       <c r="R17" s="6"/>
     </row>
-    <row r="18" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>100</v>
       </c>
@@ -2414,7 +2365,7 @@
       </c>
       <c r="R18" s="6"/>
     </row>
-    <row r="19" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>104</v>
       </c>
@@ -2451,7 +2402,7 @@
       </c>
       <c r="R19" s="6"/>
     </row>
-    <row r="20" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>108</v>
       </c>
@@ -2485,11 +2436,11 @@
       </c>
       <c r="R20" s="6"/>
     </row>
-    <row r="21" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>112</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C21" t="s">
@@ -2528,7 +2479,7 @@
       </c>
       <c r="R21" s="6"/>
     </row>
-    <row r="22" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>116</v>
       </c>
@@ -2565,7 +2516,7 @@
       </c>
       <c r="R22" s="6"/>
     </row>
-    <row r="23" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>121</v>
       </c>
@@ -2602,7 +2553,7 @@
       </c>
       <c r="R23" s="6"/>
     </row>
-    <row r="24" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>126</v>
       </c>
@@ -2639,7 +2590,7 @@
       </c>
       <c r="R24" s="6"/>
     </row>
-    <row r="25" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>131</v>
       </c>
@@ -2676,7 +2627,7 @@
       </c>
       <c r="R25" s="6"/>
     </row>
-    <row r="26" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>136</v>
       </c>
@@ -2713,7 +2664,7 @@
       </c>
       <c r="R26" s="6"/>
     </row>
-    <row r="27" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>140</v>
       </c>
@@ -2747,7 +2698,7 @@
       </c>
       <c r="R27" s="6"/>
     </row>
-    <row r="28" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>143</v>
       </c>
@@ -2787,7 +2738,7 @@
       </c>
       <c r="R28" s="6"/>
     </row>
-    <row r="29" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>148</v>
       </c>
@@ -2821,7 +2772,7 @@
       </c>
       <c r="R29" s="6"/>
     </row>
-    <row r="30" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>152</v>
       </c>
@@ -2858,11 +2809,11 @@
       </c>
       <c r="R30" s="6"/>
     </row>
-    <row r="31" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>157</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="10" t="s">
         <v>10</v>
       </c>
       <c r="C31" t="s">
@@ -2898,7 +2849,7 @@
       </c>
       <c r="R31" s="6"/>
     </row>
-    <row r="32" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>161</v>
       </c>
@@ -2935,7 +2886,7 @@
       </c>
       <c r="R32" s="6"/>
     </row>
-    <row r="33" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>165</v>
       </c>
@@ -2969,7 +2920,7 @@
       </c>
       <c r="R33" s="6"/>
     </row>
-    <row r="34" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>169</v>
       </c>
@@ -3006,7 +2957,7 @@
       </c>
       <c r="R34" s="6"/>
     </row>
-    <row r="35" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>173</v>
       </c>
@@ -3043,7 +2994,7 @@
       </c>
       <c r="R35" s="6"/>
     </row>
-    <row r="36" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>177</v>
       </c>
@@ -3077,7 +3028,7 @@
       </c>
       <c r="R36" s="6"/>
     </row>
-    <row r="37" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>180</v>
       </c>
@@ -3111,7 +3062,7 @@
       </c>
       <c r="R37" s="6"/>
     </row>
-    <row r="38" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>184</v>
       </c>
@@ -3145,7 +3096,7 @@
       </c>
       <c r="R38" s="6"/>
     </row>
-    <row r="39" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>187</v>
       </c>
@@ -3182,7 +3133,7 @@
       </c>
       <c r="R39" s="6"/>
     </row>
-    <row r="40" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>192</v>
       </c>
@@ -3216,7 +3167,7 @@
       </c>
       <c r="R40" s="6"/>
     </row>
-    <row r="41" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>196</v>
       </c>
@@ -3250,7 +3201,7 @@
       </c>
       <c r="R41" s="6"/>
     </row>
-    <row r="42" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>200</v>
       </c>
@@ -3284,7 +3235,7 @@
       </c>
       <c r="R42" s="6"/>
     </row>
-    <row r="43" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>204</v>
       </c>
@@ -3321,7 +3272,7 @@
       </c>
       <c r="R43" s="6"/>
     </row>
-    <row r="44" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>208</v>
       </c>
@@ -3358,7 +3309,7 @@
       </c>
       <c r="R44" s="6"/>
     </row>
-    <row r="45" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>211</v>
       </c>
@@ -3395,7 +3346,7 @@
       </c>
       <c r="R45" s="6"/>
     </row>
-    <row r="46" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>215</v>
       </c>
@@ -3429,7 +3380,7 @@
       </c>
       <c r="R46" s="6"/>
     </row>
-    <row r="47" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>219</v>
       </c>
@@ -3466,7 +3417,7 @@
       </c>
       <c r="R47" s="6"/>
     </row>
-    <row r="48" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>224</v>
       </c>
@@ -3503,7 +3454,7 @@
       </c>
       <c r="R48" s="6"/>
     </row>
-    <row r="49" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>229</v>
       </c>
@@ -3540,7 +3491,7 @@
       </c>
       <c r="R49" s="6"/>
     </row>
-    <row r="50" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>234</v>
       </c>
@@ -3574,8 +3525,8 @@
       </c>
       <c r="R50" s="6"/>
     </row>
-    <row r="51" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" s="11" t="s">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A51" s="10" t="s">
         <v>91</v>
       </c>
       <c r="B51" t="s">
@@ -3603,12 +3554,12 @@
         <v>8</v>
       </c>
       <c r="J51" s="6"/>
-      <c r="M51" s="10"/>
+      <c r="M51" s="7"/>
       <c r="Q51" s="8"/>
       <c r="R51" s="6"/>
     </row>
-    <row r="52" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" s="11" t="s">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A52" s="10" t="s">
         <v>91</v>
       </c>
       <c r="B52" t="s">
@@ -3633,12 +3584,12 @@
         <v>8</v>
       </c>
       <c r="J52" s="6"/>
-      <c r="M52" s="10"/>
+      <c r="M52" s="7"/>
       <c r="Q52" s="8"/>
       <c r="R52" s="6"/>
     </row>
-    <row r="53" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A53" s="11" t="s">
+    <row r="53" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A53" s="10" t="s">
         <v>91</v>
       </c>
       <c r="B53" t="s">
@@ -3663,12 +3614,12 @@
         <v>8</v>
       </c>
       <c r="J53" s="6"/>
-      <c r="M53" s="10"/>
+      <c r="M53" s="7"/>
       <c r="Q53" s="8"/>
       <c r="R53" s="6"/>
     </row>
-    <row r="54" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A54" s="11" t="s">
+    <row r="54" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A54" s="10" t="s">
         <v>91</v>
       </c>
       <c r="B54" t="s">
@@ -3693,12 +3644,12 @@
         <v>8</v>
       </c>
       <c r="J54" s="6"/>
-      <c r="M54" s="10"/>
+      <c r="M54" s="7"/>
       <c r="Q54" s="8"/>
       <c r="R54" s="6"/>
     </row>
-    <row r="55" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A55" s="11" t="s">
+    <row r="55" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A55" s="10" t="s">
         <v>91</v>
       </c>
       <c r="C55" t="s">
@@ -3720,12 +3671,12 @@
         <v>10</v>
       </c>
       <c r="J55" s="6"/>
-      <c r="M55" s="10"/>
+      <c r="M55" s="7"/>
       <c r="Q55" s="8"/>
       <c r="R55" s="6"/>
     </row>
-    <row r="56" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A56" s="11" t="s">
+    <row r="56" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A56" s="10" t="s">
         <v>91</v>
       </c>
       <c r="B56" t="s">
@@ -3750,12 +3701,12 @@
         <v>8</v>
       </c>
       <c r="J56" s="6"/>
-      <c r="M56" s="10"/>
+      <c r="M56" s="7"/>
       <c r="Q56" s="8"/>
       <c r="R56" s="6"/>
     </row>
-    <row r="57" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A57" s="11" t="s">
+    <row r="57" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A57" s="10" t="s">
         <v>263</v>
       </c>
       <c r="B57" t="s">
@@ -3783,15 +3734,15 @@
         <v>9</v>
       </c>
       <c r="J57" s="6"/>
-      <c r="M57" s="10"/>
+      <c r="M57" s="7"/>
       <c r="Q57" s="8"/>
       <c r="R57" s="6"/>
     </row>
-    <row r="58" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="11" t="s">
+    <row r="58" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A58" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C58" t="s">
@@ -3816,15 +3767,15 @@
         <v>12</v>
       </c>
       <c r="J58" s="6"/>
-      <c r="M58" s="10"/>
+      <c r="M58" s="7"/>
       <c r="Q58" s="8"/>
       <c r="R58" s="6"/>
     </row>
-    <row r="59" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A59" s="11" t="s">
+    <row r="59" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A59" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="10" t="s">
         <v>9</v>
       </c>
       <c r="C59" t="s">
@@ -3849,15 +3800,15 @@
         <v>8</v>
       </c>
       <c r="J59" s="6"/>
-      <c r="M59" s="10"/>
+      <c r="M59" s="7"/>
       <c r="Q59" s="8"/>
       <c r="R59" s="6"/>
     </row>
-    <row r="60" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A60" s="11" t="s">
+    <row r="60" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A60" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="B60" s="11" t="s">
+      <c r="B60" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C60" t="s">
@@ -3882,15 +3833,15 @@
         <v>14</v>
       </c>
       <c r="J60" s="6"/>
-      <c r="M60" s="10"/>
+      <c r="M60" s="7"/>
       <c r="Q60" s="8"/>
       <c r="R60" s="6"/>
     </row>
-    <row r="61" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="11" t="s">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A61" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B61" s="11" t="s">
+      <c r="B61" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C61" t="s">
@@ -3915,15 +3866,15 @@
         <v>16</v>
       </c>
       <c r="J61" s="6"/>
-      <c r="M61" s="10"/>
+      <c r="M61" s="7"/>
       <c r="Q61" s="8"/>
       <c r="R61" s="6"/>
     </row>
-    <row r="62" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A62" s="11" t="s">
+    <row r="62" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A62" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C62" t="s">
@@ -3948,15 +3899,15 @@
         <v>12</v>
       </c>
       <c r="J62" s="6"/>
-      <c r="M62" s="10"/>
+      <c r="M62" s="7"/>
       <c r="Q62" s="8"/>
       <c r="R62" s="6"/>
     </row>
-    <row r="63" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A63" s="11" t="s">
+    <row r="63" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A63" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C63" t="s">
@@ -3981,15 +3932,15 @@
         <v>11</v>
       </c>
       <c r="J63" s="6"/>
-      <c r="M63" s="10"/>
+      <c r="M63" s="7"/>
       <c r="Q63" s="8"/>
       <c r="R63" s="6"/>
     </row>
-    <row r="64" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A64" s="11" t="s">
+    <row r="64" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A64" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="B64" s="11" t="s">
+      <c r="B64" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C64" t="s">
@@ -4011,15 +3962,15 @@
         <v>292</v>
       </c>
       <c r="J64" s="6"/>
-      <c r="M64" s="10"/>
+      <c r="M64" s="7"/>
       <c r="Q64" s="8"/>
       <c r="R64" s="6"/>
     </row>
-    <row r="65" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A65" s="11" t="s">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A65" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" t="s">
         <v>7</v>
       </c>
       <c r="C65" t="s">
@@ -4041,15 +3992,15 @@
         <v>295</v>
       </c>
       <c r="J65" s="6"/>
-      <c r="M65" s="10"/>
+      <c r="M65" s="7"/>
       <c r="Q65" s="8"/>
       <c r="R65" s="6"/>
     </row>
-    <row r="66" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A66" s="11" t="s">
+    <row r="66" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A66" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="B66" s="11" t="s">
+      <c r="B66" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C66" t="s">
@@ -4074,15 +4025,15 @@
         <v>7</v>
       </c>
       <c r="J66" s="6"/>
-      <c r="M66" s="10"/>
+      <c r="M66" s="7"/>
       <c r="Q66" s="8"/>
       <c r="R66" s="6"/>
     </row>
-    <row r="67" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="11" t="s">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A67" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C67" t="s">
@@ -4104,15 +4055,15 @@
         <v>300</v>
       </c>
       <c r="J67" s="6"/>
-      <c r="M67" s="10"/>
+      <c r="M67" s="7"/>
       <c r="Q67" s="8"/>
       <c r="R67" s="6"/>
     </row>
-    <row r="68" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A68" s="11" t="s">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A68" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B68" s="11" t="s">
+      <c r="B68" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C68" t="s">
@@ -4137,15 +4088,15 @@
         <v>10</v>
       </c>
       <c r="J68" s="6"/>
-      <c r="M68" s="10"/>
+      <c r="M68" s="7"/>
       <c r="Q68" s="8"/>
       <c r="R68" s="6"/>
     </row>
-    <row r="69" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A69" s="11" t="s">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A69" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="B69" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C69" t="s">
@@ -4170,15 +4121,15 @@
         <v>11</v>
       </c>
       <c r="J69" s="6"/>
-      <c r="M69" s="10"/>
+      <c r="M69" s="7"/>
       <c r="Q69" s="8"/>
       <c r="R69" s="6"/>
     </row>
-    <row r="70" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A70" s="11" t="s">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A70" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="B70" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C70" t="s">
@@ -4203,15 +4154,15 @@
         <v>3</v>
       </c>
       <c r="J70" s="6"/>
-      <c r="M70" s="10"/>
+      <c r="M70" s="7"/>
       <c r="Q70" s="8"/>
       <c r="R70" s="6"/>
     </row>
-    <row r="71" spans="1:18" ht="32" x14ac:dyDescent="0.2">
-      <c r="A71" s="11" t="s">
+    <row r="71" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A71" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="B71" s="11" t="s">
+      <c r="B71" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C71" t="s">
@@ -4236,15 +4187,15 @@
         <v>4</v>
       </c>
       <c r="J71" s="6"/>
-      <c r="M71" s="10"/>
+      <c r="M71" s="7"/>
       <c r="Q71" s="8"/>
       <c r="R71" s="6"/>
     </row>
-    <row r="72" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A72" s="11" t="s">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A72" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="B72" s="11" t="s">
+      <c r="B72" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C72" t="s">
@@ -4269,79 +4220,65 @@
         <v>8</v>
       </c>
       <c r="J72" s="6"/>
-      <c r="M72" s="10"/>
+      <c r="M72" s="7"/>
       <c r="Q72" s="8"/>
       <c r="R72" s="6"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A6:R9 A11:R11 A10:G10 A13:R50 A12:G12 I12:R12 J10:R10">
-    <cfRule type="expression" dxfId="21" priority="13" stopIfTrue="1">
+  <conditionalFormatting sqref="A70:A71">
+    <cfRule type="expression" dxfId="17" priority="1" stopIfTrue="1">
+      <formula>$R70="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="2">
+      <formula>$O70="Nein"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="3">
+      <formula>$J70="TODO"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="4">
+      <formula>$J70="Abweichung"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A6:R9 A10:G10 J10:R10 A11:R11 A12:G12 I12:R12 A13:R50">
+    <cfRule type="expression" dxfId="13" priority="13" stopIfTrue="1">
       <formula>$R6="✓"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="14">
+    <cfRule type="expression" dxfId="12" priority="14">
       <formula>$O6="Nein"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="15">
+    <cfRule type="expression" dxfId="11" priority="15">
       <formula>$J6="TODO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="16">
+    <cfRule type="expression" dxfId="10" priority="16">
       <formula>$J6="Abweichung"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:I12">
-    <cfRule type="expression" dxfId="17" priority="21" stopIfTrue="1">
-      <formula>$R10="✓"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="22">
-      <formula>$O10="Nein"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="23">
-      <formula>$J10="TODO"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="24">
-      <formula>$J10="Abweichung"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A70">
-    <cfRule type="expression" dxfId="11" priority="9" stopIfTrue="1">
-      <formula>$R70="✓"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="10">
-      <formula>$O70="Nein"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="11">
-      <formula>$J70="TODO"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="12">
-      <formula>$J70="Abweichung"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C71">
-    <cfRule type="expression" dxfId="7" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="5" stopIfTrue="1">
       <formula>$R71="✓"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>$O71="Nein"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>$J71="TODO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>$J71="Abweichung"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A71">
-    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
-      <formula>$R71="✓"</formula>
+  <conditionalFormatting sqref="H12:I12">
+    <cfRule type="expression" dxfId="5" priority="21" stopIfTrue="1">
+      <formula>$R10="✓"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>$O71="Nein"</formula>
+    <cfRule type="expression" dxfId="4" priority="22">
+      <formula>$O10="Nein"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>$J71="TODO"</formula>
+    <cfRule type="expression" dxfId="3" priority="23">
+      <formula>$J10="TODO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>$J71="Abweichung"</formula>
+    <cfRule type="expression" dxfId="2" priority="24">
+      <formula>$J10="Abweichung"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4403,14 +4340,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667488DC-0E11-499F-BE9E-61EB87B6EDEE}">
   <dimension ref="A1:C46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="39.1640625" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="39.1328125" customWidth="1"/>
+    <col min="2" max="2" width="24.796875" customWidth="1"/>
     <col min="3" max="3" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>43</v>
       </c>
@@ -4421,7 +4358,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="str">
         <f>Literatur!A6</f>
         <v>stamm2021fehlenderblick</v>
@@ -4431,7 +4368,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="str">
         <f>Literatur!A7</f>
         <v>kellerkoller2021hellekoepfe</v>
@@ -4441,7 +4378,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="str">
         <f>Literatur!A8</f>
         <v>kellerkoller2009begabte</v>
@@ -4451,7 +4388,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="str">
         <f>Literatur!A9</f>
         <v>maehler2018diagnostik</v>
@@ -4461,7 +4398,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="str">
         <f>Literatur!A10</f>
         <v>preckel2013hochbegabung</v>
@@ -4471,7 +4408,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="str">
         <f>Literatur!A11</f>
         <v>muelleroppliger2021handbuch</v>
@@ -4481,7 +4418,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="str">
         <f>Literatur!A12</f>
         <v>trautmann2016einfuehrung</v>
@@ -4491,7 +4428,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="str">
         <f>Literatur!A13</f>
         <v>reutlinger2015hochbegabung</v>
@@ -4501,7 +4438,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="str">
         <f>Literatur!A14</f>
         <v>ipege2009professionelle</v>
@@ -4511,7 +4448,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="str">
         <f>Literatur!A15</f>
         <v>uslucan2012begabung</v>
@@ -4521,7 +4458,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="str">
         <f>Literatur!A16</f>
         <v>stamm2014handbuch</v>
@@ -4531,7 +4468,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="str">
         <f>Literatur!A17</f>
         <v>webb2020doppeldiagnosen</v>
@@ -4541,7 +4478,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="str">
         <f>Literatur!A18</f>
         <v>rosebrock2010grundlagen</v>
@@ -4551,7 +4488,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" t="str">
         <f>Literatur!A19</f>
         <v>gold2018lesenkannmanlernen</v>
@@ -4561,7 +4498,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="str">
         <f>Literatur!A20</f>
         <v>lehwald2017motivation</v>
@@ -4571,7 +4508,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="str">
         <f>Literatur!A21</f>
         <v>fischer2020begabungsfoerderung</v>
@@ -4581,7 +4518,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="str">
         <f>Literatur!A22</f>
         <v>sturm2016graphomotorik</v>
@@ -4591,7 +4528,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="str">
         <f>Literatur!A23</f>
         <v>grossrieder2010anerkennung</v>
@@ -4601,7 +4538,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="str">
         <f>Literatur!A24</f>
         <v>kuhl2019diversitaet</v>
@@ -4611,7 +4548,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="str">
         <f>Literatur!A25</f>
         <v>behrensen2019inklusive</v>
@@ -4621,7 +4558,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="str">
         <f>Literatur!A26</f>
         <v>booth2019index</v>
@@ -4631,7 +4568,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="str">
         <f>Literatur!A27</f>
         <v>stamm2012migranten</v>
@@ -4641,7 +4578,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="str">
         <f>Literatur!A28</f>
         <v>kappus2010migration</v>
@@ -4651,7 +4588,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="str">
         <f>Literatur!A29</f>
         <v>buholzer2010allegleich</v>
@@ -4661,7 +4598,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="str">
         <f>Literatur!A30</f>
         <v>weigand2021separativ</v>
@@ -4671,7 +4608,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="str">
         <f>Literatur!A31</f>
         <v>sedmak2021bildungsgerechtigkeit</v>
@@ -4681,7 +4618,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="str">
         <f>Literatur!A32</f>
         <v>muelleroppliger2021plurale</v>
@@ -4691,7 +4628,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" t="str">
         <f>Literatur!A33</f>
         <v>unger2010begabungsfoerderung</v>
@@ -4701,7 +4638,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" t="str">
         <f>Literatur!A34</f>
         <v>brunner2021hochbegabung</v>
@@ -4711,7 +4648,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" t="str">
         <f>Literatur!A35</f>
         <v>burow2021positive</v>
@@ -4721,7 +4658,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" t="str">
         <f>Literatur!A36</f>
         <v>burow2020future</v>
@@ -4731,7 +4668,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A33" t="str">
         <f>Literatur!A37</f>
         <v>leikhof2021jugendliche</v>
@@ -4741,7 +4678,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A34" t="str">
         <f>Literatur!A38</f>
         <v>kosoroklabhart2021voneltern</v>
@@ -4751,7 +4688,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" t="str">
         <f>Literatur!A39</f>
         <v>macha2019gender</v>
@@ -4761,7 +4698,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A36" t="str">
         <f>Literatur!A40</f>
         <v>bfs2022migration</v>
@@ -4771,7 +4708,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" t="str">
         <f>Literatur!A41</f>
         <v>erzinger2023pisa</v>
@@ -4781,7 +4718,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A38" t="str">
         <f>Literatur!A42</f>
         <v>stamm2014mirage</v>
@@ -4791,7 +4728,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" t="str">
         <f>Literatur!A43</f>
         <v>stern2025intelligenz</v>
@@ -4801,7 +4738,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" t="str">
         <f>Literatur!A44</f>
         <v>kellerkoller2011erkennen</v>
@@ -4811,7 +4748,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" t="str">
         <f>Literatur!A45</f>
         <v>lemas2023begriffsklaerung</v>
@@ -4821,7 +4758,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A42" t="str">
         <f>Literatur!A46</f>
         <v>dvs2025bbf</v>
@@ -4831,7 +4768,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" t="str">
         <f>Literatur!A47</f>
         <v>mun2020identifying</v>
@@ -4841,7 +4778,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A44" t="str">
         <f>Literatur!A48</f>
         <v>gubbins2020promising</v>
@@ -4851,7 +4788,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A45" t="str">
         <f>Literatur!A49</f>
         <v>alhroub2021utility</v>
@@ -4861,7 +4798,7 @@
         <v>TODO</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" t="str">
         <f>Literatur!A50</f>
         <v>alodat2025equitable</v>
@@ -4873,10 +4810,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C46">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>$C2="OK"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>$C2="NICHT ZITIERT"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4890,9 +4827,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{918AD35A-3B21-4D39-80D3-20FA217C7AB6}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4915,7 +4852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -4938,7 +4875,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4961,7 +4898,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -4981,7 +4918,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -4998,7 +4935,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -5012,7 +4949,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>12</v>
       </c>

</xml_diff>